<commit_message>
Fixed `normalization_layer_test_perf_report.xlsx` column names (#496)
`normalization_layer_test_perf_report.xlsx` was regenerated with the CPU
process and thread information changes made last week and pushed to
`main`. However, some of the column names in the sheets were wrong which
are fixed in `feat/add_overlapping_kernel_info_to_report`. However, now
the tests are failing for this PR since the column names of
`normalization_layer_test_perf_report.xlsx` that the test generates
don't match the same report in the repo.
I'm updating `normalization_layer_test_perf_report.xlsx` with the
changes made in `feat/add_overlapping_kernel_info_to_report`.
</commit_message>
<xml_diff>
--- a/tests/traces/perf_model/normalization/normalization_layer_test_perf_report.xlsx
+++ b/tests/traces/perf_model/normalization/normalization_layer_test_perf_report.xlsx
@@ -8870,102 +8870,102 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>process_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>process_label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>thread_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>param: op_shape</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>param: dtype_in_out</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>param: stride_input</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>param: stride_output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>GFLOPS_first</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Data Moved (MB)_first</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>FLOPS/Byte_first</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>TB/s_mean</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>TB/s_median</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>TB/s_std</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>TB/s_min</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>TB/s_max</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_mean</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_median</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_std</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_min</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_max</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>process_name_first</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>process_label_first</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>thread_name_first</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -9052,77 +9052,77 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>(8, 16)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>('float', 'float')</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>(16, 1)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>(0, 1)</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="I2" t="n">
         <v>1.28e-07</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>0.0009765625</v>
       </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
         <v>0.125</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L2" t="n">
         <v>0.0003172617769375312</v>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>0.0002957212386351248</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>9.634005023826169e-05</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>0.0002262543963750135</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>0.000491827392120075</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>3.96577221171914e-05</v>
       </c>
-      <c r="O2" t="n">
+      <c r="R2" t="n">
         <v>3.69651548293906e-05</v>
       </c>
-      <c r="P2" t="n">
+      <c r="S2" t="n">
         <v>1.204250627978271e-05</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="T2" t="n">
         <v>2.828179954687669e-05</v>
       </c>
-      <c r="R2" t="n">
+      <c r="U2" t="n">
         <v>6.147842401500938e-05</v>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -9206,112 +9206,112 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>process_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>process_label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>thread_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>param: shape_in1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>param: shape_in2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>param: dtype_in1_in2_out</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>param: stride_input1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>param: stride_input2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>param: stride_output</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>GFLOPS_first</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Data Moved (MB)_first</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>FLOPS/Byte_first</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>TB/s_mean</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>TB/s_median</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>TB/s_std</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>TB/s_min</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>TB/s_max</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_mean</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_median</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_std</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_min</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_max</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>process_name_first</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>process_label_first</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>thread_name_first</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -9398,87 +9398,87 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>(16,)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>(16,)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>('float', 'float', None)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>(1,)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>(1,)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
         <v>1.6e-08</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L2" t="n">
         <v>0.00018310546875</v>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>0.08333333333333333</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>0.0001020163951277465</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>0.0001009906255499077</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>4.268934582028177e-06</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>9.786361373817821e-05</v>
       </c>
-      <c r="O2" t="n">
+      <c r="R2" t="n">
         <v>0.0001090146936512337</v>
       </c>
-      <c r="P2" t="n">
+      <c r="S2" t="n">
         <v>8.501366260645541e-06</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="T2" t="n">
         <v>8.415885462492306e-06</v>
       </c>
-      <c r="R2" t="n">
+      <c r="U2" t="n">
         <v>3.557445485023487e-07</v>
       </c>
-      <c r="S2" t="n">
+      <c r="V2" t="n">
         <v>8.155301144848183e-06</v>
       </c>
-      <c r="T2" t="n">
+      <c r="W2" t="n">
         <v>9.084557804269476e-06</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -9548,87 +9548,87 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>()</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>('long int', 'long int', None)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="K3" t="n">
         <v>1e-09</v>
       </c>
-      <c r="I3" t="n">
+      <c r="L3" t="n">
         <v>2.288818359375e-05</v>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
         <v>0.04166666666666666</v>
       </c>
-      <c r="K3" t="n">
+      <c r="N3" t="n">
         <v>8.159373148075394e-06</v>
       </c>
-      <c r="L3" t="n">
+      <c r="O3" t="n">
         <v>6.712597892214445e-06</v>
       </c>
-      <c r="M3" t="n">
+      <c r="P3" t="n">
         <v>3.242418453072257e-06</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>5.211748489025555e-06</v>
       </c>
-      <c r="O3" t="n">
+      <c r="R3" t="n">
         <v>1.275350285417748e-05</v>
       </c>
-      <c r="P3" t="n">
+      <c r="S3" t="n">
         <v>3.399738811698081e-07</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="T3" t="n">
         <v>2.796915788422685e-07</v>
       </c>
-      <c r="R3" t="n">
+      <c r="U3" t="n">
         <v>1.351007688780107e-07</v>
       </c>
-      <c r="S3" t="n">
+      <c r="V3" t="n">
         <v>2.171561870427314e-07</v>
       </c>
-      <c r="T3" t="n">
+      <c r="W3" t="n">
         <v>5.313959522573949e-07</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr">
@@ -9694,87 +9694,87 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>(16, 32, 32)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>(16, 32, 32)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>('float', 'float', None)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>(1024, 32, 1)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>(1024, 32, 1)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="K4" t="n">
         <v>1.6384e-05</v>
       </c>
-      <c r="I4" t="n">
+      <c r="L4" t="n">
         <v>0.1875</v>
       </c>
-      <c r="J4" t="n">
+      <c r="M4" t="n">
         <v>0.08333333333333333</v>
       </c>
-      <c r="K4" t="n">
+      <c r="N4" t="n">
         <v>0.04795802613051017</v>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>0.0480332236803435</v>
       </c>
-      <c r="M4" t="n">
+      <c r="P4" t="n">
         <v>0.003386136466877823</v>
       </c>
-      <c r="N4" t="n">
+      <c r="Q4" t="n">
         <v>0.04463509411373463</v>
       </c>
-      <c r="O4" t="n">
+      <c r="R4" t="n">
         <v>0.05113056304761905</v>
       </c>
-      <c r="P4" t="n">
+      <c r="S4" t="n">
         <v>0.003996502177542514</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="T4" t="n">
         <v>0.004002768640028624</v>
       </c>
-      <c r="R4" t="n">
+      <c r="U4" t="n">
         <v>0.0002821780389064852</v>
       </c>
-      <c r="S4" t="n">
+      <c r="V4" t="n">
         <v>0.003719591176144552</v>
       </c>
-      <c r="T4" t="n">
+      <c r="W4" t="n">
         <v>0.004260880253968253</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -9844,87 +9844,87 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>(32, 32)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>(32, 32)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>('float', 'float', None)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>(32, 1)</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>(32, 1)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="K5" t="n">
         <v>1.024e-06</v>
       </c>
-      <c r="I5" t="n">
+      <c r="L5" t="n">
         <v>0.01171875</v>
       </c>
-      <c r="J5" t="n">
+      <c r="M5" t="n">
         <v>0.08333333333333333</v>
       </c>
-      <c r="K5" t="n">
+      <c r="N5" t="n">
         <v>0.005466037708706859</v>
       </c>
-      <c r="L5" t="n">
+      <c r="O5" t="n">
         <v>0.005466037708706859</v>
       </c>
-      <c r="M5" t="n">
+      <c r="P5" t="n">
         <v>0.0006164429592976079</v>
       </c>
-      <c r="N5" t="n">
+      <c r="Q5" t="n">
         <v>0.005030146711972817</v>
       </c>
-      <c r="O5" t="n">
+      <c r="R5" t="n">
         <v>0.0059019287054409</v>
       </c>
-      <c r="P5" t="n">
+      <c r="S5" t="n">
         <v>0.0004555031423922382</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="T5" t="n">
         <v>0.0004555031423922382</v>
       </c>
-      <c r="R5" t="n">
+      <c r="U5" t="n">
         <v>5.137024660813406e-05</v>
       </c>
-      <c r="S5" t="n">
+      <c r="V5" t="n">
         <v>0.0004191788926644014</v>
       </c>
-      <c r="T5" t="n">
+      <c r="W5" t="n">
         <v>0.000491827392120075</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -9994,46 +9994,58 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>(1,)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>('long int', 'Scalar', None)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>(1,)</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="K6" t="n">
         <v>1e-09</v>
       </c>
-      <c r="I6" t="n">
+      <c r="L6" t="n">
         <v>1.9073486328125e-05</v>
       </c>
-      <c r="J6" t="n">
+      <c r="M6" t="n">
         <v>0.05</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -10041,21 +10053,9 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
@@ -10116,46 +10116,58 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>(1,)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>('long int', 'long int', None)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>(1,)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>()</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="K7" t="n">
         <v>1e-09</v>
       </c>
-      <c r="I7" t="n">
+      <c r="L7" t="n">
         <v>2.288818359375e-05</v>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>0.04166666666666666</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -10163,21 +10175,9 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr">
         <is>
@@ -10252,127 +10252,127 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>process_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>process_label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>thread_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>param: op_shape</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>param: dtype_in_out</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>param: stride_input</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>param: stride_output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>param: num_channels</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>param: has_bias</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>param: is_affine</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>param: is_training</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>param: output_mask</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>GFLOPS_first</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Data Moved (MB)_first</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>FLOPS/Byte_first</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>TB/s_mean</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>TB/s_median</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>TB/s_std</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>TB/s_min</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>TB/s_max</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_mean</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_median</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_std</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_min</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>TFLOPS/s_max</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>process_name_first</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>process_label_first</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>thread_name_first</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
@@ -10459,102 +10459,102 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>0.000655456</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>1.0003662109375</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>0.624862721171446</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>0.06029117081479473</v>
       </c>
-      <c r="O2" t="n">
+      <c r="R2" t="n">
         <v>0.06186871052394456</v>
       </c>
-      <c r="P2" t="n">
+      <c r="S2" t="n">
         <v>0.01901091404536839</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="T2" t="n">
         <v>0.02730805511770987</v>
       </c>
-      <c r="R2" t="n">
+      <c r="U2" t="n">
         <v>0.08236284476478933</v>
       </c>
-      <c r="S2" t="n">
+      <c r="V2" t="n">
         <v>0.0376737050579451</v>
       </c>
-      <c r="T2" t="n">
+      <c r="W2" t="n">
         <v>0.03865945081336047</v>
       </c>
-      <c r="U2" t="n">
+      <c r="X2" t="n">
         <v>0.01187921148234536</v>
       </c>
-      <c r="V2" t="n">
+      <c r="Y2" t="n">
         <v>0.01706378563075202</v>
       </c>
-      <c r="W2" t="n">
+      <c r="Z2" t="n">
         <v>0.05146547130314764</v>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -10624,102 +10624,102 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>16384.0</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>[True, True, True]</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="N3" t="n">
         <v>0.001179648</v>
       </c>
-      <c r="L3" t="n">
+      <c r="O3" t="n">
         <v>1.75</v>
       </c>
-      <c r="M3" t="n">
+      <c r="P3" t="n">
         <v>0.6428571428571429</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>0.05628963269412802</v>
       </c>
-      <c r="O3" t="n">
+      <c r="R3" t="n">
         <v>0.05683579419860258</v>
       </c>
-      <c r="P3" t="n">
+      <c r="S3" t="n">
         <v>0.001008475034056347</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="T3" t="n">
         <v>0.05512587657870418</v>
       </c>
-      <c r="R3" t="n">
+      <c r="U3" t="n">
         <v>0.0569072273050773</v>
       </c>
-      <c r="S3" t="n">
+      <c r="V3" t="n">
         <v>0.03618619244622515</v>
       </c>
-      <c r="T3" t="n">
+      <c r="W3" t="n">
         <v>0.03653729627053023</v>
       </c>
-      <c r="U3" t="n">
+      <c r="X3" t="n">
         <v>0.0006483053790362222</v>
       </c>
-      <c r="V3" t="n">
+      <c r="Y3" t="n">
         <v>0.03543806351488125</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Z3" t="n">
         <v>0.03658321755326398</v>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
@@ -10789,102 +10789,102 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="N4" t="n">
         <v>0.000655456</v>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>1.0003662109375</v>
       </c>
-      <c r="M4" t="n">
+      <c r="P4" t="n">
         <v>0.624862721171446</v>
       </c>
-      <c r="N4" t="n">
+      <c r="Q4" t="n">
         <v>0.07847361405809597</v>
       </c>
-      <c r="O4" t="n">
+      <c r="R4" t="n">
         <v>0.07186558594633613</v>
       </c>
-      <c r="P4" t="n">
+      <c r="S4" t="n">
         <v>0.02181711774215055</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="T4" t="n">
         <v>0.05680999814888272</v>
       </c>
-      <c r="R4" t="n">
+      <c r="U4" t="n">
         <v>0.1133891101023963</v>
       </c>
-      <c r="S4" t="n">
+      <c r="V4" t="n">
         <v>0.04903523602049969</v>
       </c>
-      <c r="T4" t="n">
+      <c r="W4" t="n">
         <v>0.04490612559300802</v>
       </c>
-      <c r="U4" t="n">
+      <c r="X4" t="n">
         <v>0.01363270356047803</v>
       </c>
-      <c r="V4" t="n">
+      <c r="Y4" t="n">
         <v>0.03549845003305566</v>
       </c>
-      <c r="W4" t="n">
+      <c r="Z4" t="n">
         <v>0.07085262788979203</v>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -10954,102 +10954,102 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>16384.0</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="N5" t="n">
         <v>0.000753664</v>
       </c>
-      <c r="L5" t="n">
+      <c r="O5" t="n">
         <v>1.375</v>
       </c>
-      <c r="M5" t="n">
+      <c r="P5" t="n">
         <v>0.5227272727272727</v>
       </c>
-      <c r="N5" t="n">
+      <c r="Q5" t="n">
         <v>0.1057710683031978</v>
       </c>
-      <c r="O5" t="n">
+      <c r="R5" t="n">
         <v>0.1083376318348772</v>
       </c>
-      <c r="P5" t="n">
+      <c r="S5" t="n">
         <v>0.01319441490156889</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="T5" t="n">
         <v>0.082553959293223</v>
       </c>
-      <c r="R5" t="n">
+      <c r="U5" t="n">
         <v>0.1176222919056724</v>
       </c>
-      <c r="S5" t="n">
+      <c r="V5" t="n">
         <v>0.05528942206758067</v>
       </c>
-      <c r="T5" t="n">
+      <c r="W5" t="n">
         <v>0.05663103482277673</v>
       </c>
-      <c r="U5" t="n">
+      <c r="X5" t="n">
         <v>0.006897080516729191</v>
       </c>
-      <c r="V5" t="n">
+      <c r="Y5" t="n">
         <v>0.04315320599418475</v>
       </c>
-      <c r="W5" t="n">
+      <c r="Z5" t="n">
         <v>0.0614843798597833</v>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -11119,102 +11119,102 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>16384.0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="N6" t="n">
         <v>0.000753664</v>
       </c>
-      <c r="L6" t="n">
+      <c r="O6" t="n">
         <v>1.375</v>
       </c>
-      <c r="M6" t="n">
+      <c r="P6" t="n">
         <v>0.5227272727272727</v>
       </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
         <v>0.1057710683031978</v>
       </c>
-      <c r="O6" t="n">
+      <c r="R6" t="n">
         <v>0.1083376318348772</v>
       </c>
-      <c r="P6" t="n">
+      <c r="S6" t="n">
         <v>0.01319441490156889</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="T6" t="n">
         <v>0.082553959293223</v>
       </c>
-      <c r="R6" t="n">
+      <c r="U6" t="n">
         <v>0.1176222919056724</v>
       </c>
-      <c r="S6" t="n">
+      <c r="V6" t="n">
         <v>0.05528942206758067</v>
       </c>
-      <c r="T6" t="n">
+      <c r="W6" t="n">
         <v>0.05663103482277673</v>
       </c>
-      <c r="U6" t="n">
+      <c r="X6" t="n">
         <v>0.006897080516729191</v>
       </c>
-      <c r="V6" t="n">
+      <c r="Y6" t="n">
         <v>0.04315320599418475</v>
       </c>
-      <c r="W6" t="n">
+      <c r="Z6" t="n">
         <v>0.0614843798597833</v>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -11284,102 +11284,102 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="N7" t="n">
         <v>0.000655456</v>
       </c>
-      <c r="L7" t="n">
+      <c r="O7" t="n">
         <v>1.0003662109375</v>
       </c>
-      <c r="M7" t="n">
+      <c r="P7" t="n">
         <v>0.624862721171446</v>
       </c>
-      <c r="N7" t="n">
+      <c r="Q7" t="n">
         <v>0.08244925142955863</v>
       </c>
-      <c r="O7" t="n">
+      <c r="R7" t="n">
         <v>0.08380426443270807</v>
       </c>
-      <c r="P7" t="n">
+      <c r="S7" t="n">
         <v>0.02125372186575851</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="T7" t="n">
         <v>0.05768561746462232</v>
       </c>
-      <c r="R7" t="n">
+      <c r="U7" t="n">
         <v>0.1158846736433272</v>
       </c>
-      <c r="S7" t="n">
+      <c r="V7" t="n">
         <v>0.05151946360682275</v>
       </c>
-      <c r="T7" t="n">
+      <c r="W7" t="n">
         <v>0.05236616071919339</v>
       </c>
-      <c r="U7" t="n">
+      <c r="X7" t="n">
         <v>0.01328065848005892</v>
       </c>
-      <c r="V7" t="n">
+      <c r="Y7" t="n">
         <v>0.03604559190139899</v>
       </c>
-      <c r="W7" t="n">
+      <c r="Z7" t="n">
         <v>0.0724120125148344</v>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -11449,102 +11449,102 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="N8" t="n">
         <v>0.000655456</v>
       </c>
-      <c r="L8" t="n">
+      <c r="O8" t="n">
         <v>1.0003662109375</v>
       </c>
-      <c r="M8" t="n">
+      <c r="P8" t="n">
         <v>0.624862721171446</v>
       </c>
-      <c r="N8" t="n">
+      <c r="Q8" t="n">
         <v>0.08244925142955863</v>
       </c>
-      <c r="O8" t="n">
+      <c r="R8" t="n">
         <v>0.08380426443270807</v>
       </c>
-      <c r="P8" t="n">
+      <c r="S8" t="n">
         <v>0.02125372186575851</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="T8" t="n">
         <v>0.05768561746462232</v>
       </c>
-      <c r="R8" t="n">
+      <c r="U8" t="n">
         <v>0.1158846736433272</v>
       </c>
-      <c r="S8" t="n">
+      <c r="V8" t="n">
         <v>0.05151946360682275</v>
       </c>
-      <c r="T8" t="n">
+      <c r="W8" t="n">
         <v>0.05236616071919339</v>
       </c>
-      <c r="U8" t="n">
+      <c r="X8" t="n">
         <v>0.01328065848005892</v>
       </c>
-      <c r="V8" t="n">
+      <c r="Y8" t="n">
         <v>0.03604559190139899</v>
       </c>
-      <c r="W8" t="n">
+      <c r="Z8" t="n">
         <v>0.0724120125148344</v>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -11614,102 +11614,102 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>16384.0</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>[True, False, False]</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="N9" t="n">
         <v>0.001179648</v>
       </c>
-      <c r="L9" t="n">
+      <c r="O9" t="n">
         <v>1.5625</v>
       </c>
-      <c r="M9" t="n">
+      <c r="P9" t="n">
         <v>0.72</v>
       </c>
-      <c r="N9" t="n">
+      <c r="Q9" t="n">
         <v>0.06680599771272798</v>
       </c>
-      <c r="O9" t="n">
+      <c r="R9" t="n">
         <v>0.06661193893554086</v>
       </c>
-      <c r="P9" t="n">
+      <c r="S9" t="n">
         <v>0.00219379562352543</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="T9" t="n">
         <v>0.06471567821944493</v>
       </c>
-      <c r="R9" t="n">
+      <c r="U9" t="n">
         <v>0.06909037598319813</v>
       </c>
-      <c r="S9" t="n">
+      <c r="V9" t="n">
         <v>0.04810031835316414</v>
       </c>
-      <c r="T9" t="n">
+      <c r="W9" t="n">
         <v>0.04796059603358942</v>
       </c>
-      <c r="U9" t="n">
+      <c r="X9" t="n">
         <v>0.001579532848938307</v>
       </c>
-      <c r="V9" t="n">
+      <c r="Y9" t="n">
         <v>0.04659528831800035</v>
       </c>
-      <c r="W9" t="n">
+      <c r="Z9" t="n">
         <v>0.04974507070790265</v>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -11779,102 +11779,102 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K10" t="n">
+      <c r="N10" t="n">
         <v>0.000655456</v>
       </c>
-      <c r="L10" t="n">
+      <c r="O10" t="n">
         <v>1.0003662109375</v>
       </c>
-      <c r="M10" t="n">
+      <c r="P10" t="n">
         <v>0.624862721171446</v>
       </c>
-      <c r="N10" t="n">
+      <c r="Q10" t="n">
         <v>0.06114965934906944</v>
       </c>
-      <c r="O10" t="n">
+      <c r="R10" t="n">
         <v>0.0737780781647091</v>
       </c>
-      <c r="P10" t="n">
+      <c r="S10" t="n">
         <v>0.02962035089441791</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="T10" t="n">
         <v>0.02730805511770987</v>
       </c>
-      <c r="R10" t="n">
+      <c r="U10" t="n">
         <v>0.08236284476478933</v>
       </c>
-      <c r="S10" t="n">
+      <c r="V10" t="n">
         <v>0.03821014253956648</v>
       </c>
-      <c r="T10" t="n">
+      <c r="W10" t="n">
         <v>0.04610117068479978</v>
       </c>
-      <c r="U10" t="n">
+      <c r="X10" t="n">
         <v>0.01850865306193904</v>
       </c>
-      <c r="V10" t="n">
+      <c r="Y10" t="n">
         <v>0.01706378563075202</v>
       </c>
-      <c r="W10" t="n">
+      <c r="Z10" t="n">
         <v>0.05146547130314764</v>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -11944,102 +11944,102 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>(1, 128, 32, 32)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>(131072, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>128.0</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K11" t="n">
+      <c r="N11" t="n">
         <v>0.000656128</v>
       </c>
-      <c r="L11" t="n">
+      <c r="O11" t="n">
         <v>1.0029296875</v>
       </c>
-      <c r="M11" t="n">
+      <c r="P11" t="n">
         <v>0.623904576436222</v>
       </c>
-      <c r="N11" t="n">
+      <c r="Q11" t="n">
         <v>0.1528552967558544</v>
       </c>
-      <c r="O11" t="n">
+      <c r="R11" t="n">
         <v>0.1386079341065403</v>
       </c>
-      <c r="P11" t="n">
+      <c r="S11" t="n">
         <v>0.1016204193338914</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="T11" t="n">
         <v>0.05695557593547534</v>
       </c>
-      <c r="R11" t="n">
+      <c r="U11" t="n">
         <v>0.2679491296342374</v>
       </c>
-      <c r="S11" t="n">
+      <c r="V11" t="n">
         <v>0.09536711917849433</v>
       </c>
-      <c r="T11" t="n">
+      <c r="W11" t="n">
         <v>0.0864781244194408</v>
       </c>
-      <c r="U11" t="n">
+      <c r="X11" t="n">
         <v>0.06340144468178278</v>
       </c>
-      <c r="V11" t="n">
+      <c r="Y11" t="n">
         <v>0.03553484447970382</v>
       </c>
-      <c r="W11" t="n">
+      <c r="Z11" t="n">
         <v>0.1671746882309032</v>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -12109,102 +12109,102 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>[True, True, True]</t>
         </is>
       </c>
-      <c r="K12" t="n">
+      <c r="N12" t="n">
         <v>0.001179648</v>
       </c>
-      <c r="L12" t="n">
+      <c r="O12" t="n">
         <v>1.50006103515625</v>
       </c>
-      <c r="M12" t="n">
+      <c r="P12" t="n">
         <v>0.749969483663588</v>
       </c>
-      <c r="N12" t="n">
+      <c r="Q12" t="n">
         <v>0.08158110778877121</v>
       </c>
-      <c r="O12" t="n">
+      <c r="R12" t="n">
         <v>0.07823573877352762</v>
       </c>
-      <c r="P12" t="n">
+      <c r="S12" t="n">
         <v>0.008789629375982646</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="T12" t="n">
         <v>0.07495536086744072</v>
       </c>
-      <c r="R12" t="n">
+      <c r="U12" t="n">
         <v>0.0915522237253453</v>
       </c>
-      <c r="S12" t="n">
+      <c r="V12" t="n">
         <v>0.06118334128504826</v>
       </c>
-      <c r="T12" t="n">
+      <c r="W12" t="n">
         <v>0.05867441661202185</v>
       </c>
-      <c r="U12" t="n">
+      <c r="X12" t="n">
         <v>0.006591953804700008</v>
       </c>
-      <c r="V12" t="n">
+      <c r="Y12" t="n">
         <v>0.05621423328757242</v>
       </c>
-      <c r="W12" t="n">
+      <c r="Z12" t="n">
         <v>0.0686613739555505</v>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -12274,102 +12274,102 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="N13" t="n">
         <v>0.000655456</v>
       </c>
-      <c r="L13" t="n">
+      <c r="O13" t="n">
         <v>1.0003662109375</v>
       </c>
-      <c r="M13" t="n">
+      <c r="P13" t="n">
         <v>0.624862721171446</v>
       </c>
-      <c r="N13" t="n">
+      <c r="Q13" t="n">
         <v>0.05943268228052002</v>
       </c>
-      <c r="O13" t="n">
+      <c r="R13" t="n">
         <v>0.05938713108862719</v>
       </c>
-      <c r="P13" t="n">
+      <c r="S13" t="n">
         <v>0.004894991042083343</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="T13" t="n">
         <v>0.05456062579367095</v>
       </c>
-      <c r="R13" t="n">
+      <c r="U13" t="n">
         <v>0.06435028995926192</v>
       </c>
-      <c r="S13" t="n">
+      <c r="V13" t="n">
         <v>0.03713726757632372</v>
       </c>
-      <c r="T13" t="n">
+      <c r="W13" t="n">
         <v>0.03710880433460496</v>
       </c>
-      <c r="U13" t="n">
+      <c r="X13" t="n">
         <v>0.003058697422666048</v>
       </c>
-      <c r="V13" t="n">
+      <c r="Y13" t="n">
         <v>0.03409290110225022</v>
       </c>
-      <c r="W13" t="n">
+      <c r="Z13" t="n">
         <v>0.04021009729211598</v>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -12439,102 +12439,102 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>(1, 128, 32, 32)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>(131072, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>128.0</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K14" t="n">
+      <c r="N14" t="n">
         <v>0.000656128</v>
       </c>
-      <c r="L14" t="n">
+      <c r="O14" t="n">
         <v>1.0029296875</v>
       </c>
-      <c r="M14" t="n">
+      <c r="P14" t="n">
         <v>0.623904576436222</v>
       </c>
-      <c r="N14" t="n">
+      <c r="Q14" t="n">
         <v>0.06165094775847439</v>
       </c>
-      <c r="O14" t="n">
+      <c r="R14" t="n">
         <v>0.06251705622478303</v>
       </c>
-      <c r="P14" t="n">
+      <c r="S14" t="n">
         <v>0.004327812281425612</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="T14" t="n">
         <v>0.05695557593547534</v>
       </c>
-      <c r="R14" t="n">
+      <c r="U14" t="n">
         <v>0.06548021111516479</v>
       </c>
-      <c r="S14" t="n">
+      <c r="V14" t="n">
         <v>0.03846430844814261</v>
       </c>
-      <c r="T14" t="n">
+      <c r="W14" t="n">
         <v>0.03900467748396273</v>
       </c>
-      <c r="U14" t="n">
+      <c r="X14" t="n">
         <v>0.002700141888338324</v>
       </c>
-      <c r="V14" t="n">
+      <c r="Y14" t="n">
         <v>0.03553484447970382</v>
       </c>
-      <c r="W14" t="n">
+      <c r="Z14" t="n">
         <v>0.04085340338076128</v>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -12604,102 +12604,102 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>1024.0</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>[True, True]</t>
         </is>
       </c>
-      <c r="K15" t="n">
+      <c r="N15" t="n">
         <v>0.00131072</v>
       </c>
-      <c r="L15" t="n">
+      <c r="O15" t="n">
         <v>1.5078125</v>
       </c>
-      <c r="M15" t="n">
+      <c r="P15" t="n">
         <v>0.8290155440414507</v>
       </c>
-      <c r="N15" t="n">
+      <c r="Q15" t="n">
         <v>0.09662045428134391</v>
       </c>
-      <c r="O15" t="n">
+      <c r="R15" t="n">
         <v>0.09795210357866714</v>
       </c>
-      <c r="P15" t="n">
+      <c r="S15" t="n">
         <v>0.005130784259081977</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="T15" t="n">
         <v>0.09095513168539326</v>
       </c>
-      <c r="R15" t="n">
+      <c r="U15" t="n">
         <v>0.1009541275799713</v>
       </c>
-      <c r="S15" t="n">
+      <c r="V15" t="n">
         <v>0.08009985847158045</v>
       </c>
-      <c r="T15" t="n">
+      <c r="W15" t="n">
         <v>0.08120381643827329</v>
       </c>
-      <c r="U15" t="n">
+      <c r="X15" t="n">
         <v>0.004253499903902161</v>
       </c>
-      <c r="V15" t="n">
+      <c r="Y15" t="n">
         <v>0.07540321797752809</v>
       </c>
-      <c r="W15" t="n">
+      <c r="Z15" t="n">
         <v>0.08369254099893997</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -12769,102 +12769,102 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>[True, False, False]</t>
         </is>
       </c>
-      <c r="K16" t="n">
+      <c r="N16" t="n">
         <v>0.001179648</v>
       </c>
-      <c r="L16" t="n">
+      <c r="O16" t="n">
         <v>1.50006103515625</v>
       </c>
-      <c r="M16" t="n">
+      <c r="P16" t="n">
         <v>0.749969483663588</v>
       </c>
-      <c r="N16" t="n">
+      <c r="Q16" t="n">
         <v>0.1160727043946573</v>
       </c>
-      <c r="O16" t="n">
+      <c r="R16" t="n">
         <v>0.1204695790575916</v>
       </c>
-      <c r="P16" t="n">
+      <c r="S16" t="n">
         <v>0.02471211817896858</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="T16" t="n">
         <v>0.08945727697861705</v>
       </c>
-      <c r="R16" t="n">
+      <c r="U16" t="n">
         <v>0.1382912571477634</v>
       </c>
-      <c r="S16" t="n">
+      <c r="V16" t="n">
         <v>0.08705098618229744</v>
       </c>
-      <c r="T16" t="n">
+      <c r="W16" t="n">
         <v>0.09034850800299177</v>
       </c>
-      <c r="U16" t="n">
+      <c r="X16" t="n">
         <v>0.01853333451091463</v>
       </c>
-      <c r="V16" t="n">
+      <c r="Y16" t="n">
         <v>0.06709022782560399</v>
       </c>
-      <c r="W16" t="n">
+      <c r="Z16" t="n">
         <v>0.1037142227182966</v>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -12934,102 +12934,102 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>[True]</t>
         </is>
       </c>
-      <c r="K17" t="n">
+      <c r="N17" t="n">
         <v>0.001179648</v>
       </c>
-      <c r="L17" t="n">
+      <c r="O17" t="n">
         <v>1.500244140625</v>
       </c>
-      <c r="M17" t="n">
+      <c r="P17" t="n">
         <v>0.7498779495524817</v>
       </c>
-      <c r="N17" t="n">
+      <c r="Q17" t="n">
         <v>0.13861462663244</v>
       </c>
-      <c r="O17" t="n">
+      <c r="R17" t="n">
         <v>0.138284391793287</v>
       </c>
-      <c r="P17" t="n">
+      <c r="S17" t="n">
         <v>0.001021216688976221</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="T17" t="n">
         <v>0.1377993909324209</v>
       </c>
-      <c r="R17" t="n">
+      <c r="U17" t="n">
         <v>0.139760097171612</v>
       </c>
-      <c r="S17" t="n">
+      <c r="V17" t="n">
         <v>0.1039440519971169</v>
       </c>
-      <c r="T17" t="n">
+      <c r="W17" t="n">
         <v>0.1036964161730621</v>
       </c>
-      <c r="U17" t="n">
+      <c r="X17" t="n">
         <v>0.0007657878767782663</v>
       </c>
-      <c r="V17" t="n">
+      <c r="Y17" t="n">
         <v>0.1033327247219846</v>
       </c>
-      <c r="W17" t="n">
+      <c r="Z17" t="n">
         <v>0.104803015096304</v>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -13099,102 +13099,102 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>1024.0</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K18" t="n">
+      <c r="N18" t="n">
         <v>0.0005245440000000001</v>
       </c>
-      <c r="L18" t="n">
+      <c r="O18" t="n">
         <v>1.00390625</v>
       </c>
-      <c r="M18" t="n">
+      <c r="P18" t="n">
         <v>0.4982976653696498</v>
       </c>
-      <c r="N18" t="n">
+      <c r="Q18" t="n">
         <v>0.2345369704960928</v>
       </c>
-      <c r="O18" t="n">
+      <c r="R18" t="n">
         <v>0.2479439085124426</v>
       </c>
-      <c r="P18" t="n">
+      <c r="S18" t="n">
         <v>0.02585868594391625</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="T18" t="n">
         <v>0.1904312566027736</v>
       </c>
-      <c r="R18" t="n">
+      <c r="U18" t="n">
         <v>0.2551328113609468</v>
       </c>
-      <c r="S18" t="n">
+      <c r="V18" t="n">
         <v>0.1168692248410735</v>
       </c>
-      <c r="T18" t="n">
+      <c r="W18" t="n">
         <v>0.1235498707543762</v>
       </c>
-      <c r="U18" t="n">
+      <c r="X18" t="n">
         <v>0.01288532283538044</v>
       </c>
-      <c r="V18" t="n">
+      <c r="Y18" t="n">
         <v>0.09489145057857082</v>
       </c>
-      <c r="W18" t="n">
+      <c r="Z18" t="n">
         <v>0.127132084260355</v>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -13264,102 +13264,102 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>(1, 128, 32, 32)</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>(131072, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>128.0</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>[True]</t>
         </is>
       </c>
-      <c r="K19" t="n">
+      <c r="N19" t="n">
         <v>0.001179648</v>
       </c>
-      <c r="L19" t="n">
+      <c r="O19" t="n">
         <v>1.501953125</v>
       </c>
-      <c r="M19" t="n">
+      <c r="P19" t="n">
         <v>0.7490247074122237</v>
       </c>
-      <c r="N19" t="n">
+      <c r="Q19" t="n">
         <v>0.241821376849506</v>
       </c>
-      <c r="O19" t="n">
+      <c r="R19" t="n">
         <v>0.2488365820089493</v>
       </c>
-      <c r="P19" t="n">
+      <c r="S19" t="n">
         <v>0.0297823893140027</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="T19" t="n">
         <v>0.2091576276506063</v>
       </c>
-      <c r="R19" t="n">
+      <c r="U19" t="n">
         <v>0.2674699208889626</v>
       </c>
-      <c r="S19" t="n">
+      <c r="V19" t="n">
         <v>0.1811301860407223</v>
       </c>
-      <c r="T19" t="n">
+      <c r="W19" t="n">
         <v>0.186384748032711</v>
       </c>
-      <c r="U19" t="n">
+      <c r="X19" t="n">
         <v>0.0223077454419578</v>
       </c>
-      <c r="V19" t="n">
+      <c r="Y19" t="n">
         <v>0.1566642308540302</v>
       </c>
-      <c r="W19" t="n">
+      <c r="Z19" t="n">
         <v>0.2003415792354258</v>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -13429,102 +13429,102 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>1024.0</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>[True, False]</t>
         </is>
       </c>
-      <c r="K20" t="n">
+      <c r="N20" t="n">
         <v>0.001048576</v>
       </c>
-      <c r="L20" t="n">
+      <c r="O20" t="n">
         <v>1.5078125</v>
       </c>
-      <c r="M20" t="n">
+      <c r="P20" t="n">
         <v>0.6632124352331606</v>
       </c>
-      <c r="N20" t="n">
+      <c r="Q20" t="n">
         <v>0.2734392754403918</v>
       </c>
-      <c r="O20" t="n">
+      <c r="R20" t="n">
         <v>0.2881554407760079</v>
       </c>
-      <c r="P20" t="n">
+      <c r="S20" t="n">
         <v>0.03747419808787525</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="T20" t="n">
         <v>0.2308407134811435</v>
       </c>
-      <c r="R20" t="n">
+      <c r="U20" t="n">
         <v>0.3013216720640238</v>
       </c>
-      <c r="S20" t="n">
+      <c r="V20" t="n">
         <v>0.1813483277532132</v>
       </c>
-      <c r="T20" t="n">
+      <c r="W20" t="n">
         <v>0.1911082716027409</v>
       </c>
-      <c r="U20" t="n">
+      <c r="X20" t="n">
         <v>0.0248533541722696</v>
       </c>
-      <c r="V20" t="n">
+      <c r="Y20" t="n">
         <v>0.1530964317387895</v>
       </c>
-      <c r="W20" t="n">
+      <c r="Z20" t="n">
         <v>0.199840279918109</v>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -13594,102 +13594,102 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>(8, 16, 32, 32)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>(16384, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>[True]</t>
         </is>
       </c>
-      <c r="K21" t="n">
+      <c r="N21" t="n">
         <v>0.000524336</v>
       </c>
-      <c r="L21" t="n">
+      <c r="O21" t="n">
         <v>1.00006103515625</v>
       </c>
-      <c r="M21" t="n">
+      <c r="P21" t="n">
         <v>0.5000152578577968</v>
       </c>
-      <c r="N21" t="n">
+      <c r="Q21" t="n">
         <v>0.2067490101745708</v>
       </c>
-      <c r="O21" t="n">
+      <c r="R21" t="n">
         <v>0.2094416539886874</v>
       </c>
-      <c r="P21" t="n">
+      <c r="S21" t="n">
         <v>0.01852446773236728</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="T21" t="n">
         <v>0.1870255786815292</v>
       </c>
-      <c r="R21" t="n">
+      <c r="U21" t="n">
         <v>0.2237797978534959</v>
       </c>
-      <c r="S21" t="n">
+      <c r="V21" t="n">
         <v>0.1033776596342823</v>
       </c>
-      <c r="T21" t="n">
+      <c r="W21" t="n">
         <v>0.104724022625317</v>
       </c>
-      <c r="U21" t="n">
+      <c r="X21" t="n">
         <v>0.00926251650987806</v>
       </c>
-      <c r="V21" t="n">
+      <c r="Y21" t="n">
         <v>0.09351564295044849</v>
       </c>
-      <c r="W21" t="n">
+      <c r="Z21" t="n">
         <v>0.1118933133270814</v>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -13759,102 +13759,102 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>thread 2300680 (pt_autograd_0)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
           <t>(1, 128, 32, 32)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>(131072, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>128.0</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>[True]</t>
         </is>
       </c>
-      <c r="K22" t="n">
+      <c r="N22" t="n">
         <v>0.000524672</v>
       </c>
-      <c r="L22" t="n">
+      <c r="O22" t="n">
         <v>1.00048828125</v>
       </c>
-      <c r="M22" t="n">
+      <c r="P22" t="n">
         <v>0.5001220107369448</v>
       </c>
-      <c r="N22" t="n">
+      <c r="Q22" t="n">
         <v>0.2371125493316399</v>
       </c>
-      <c r="O22" t="n">
+      <c r="R22" t="n">
         <v>0.2447632973342447</v>
       </c>
-      <c r="P22" t="n">
+      <c r="S22" t="n">
         <v>0.02942084384243977</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="T22" t="n">
         <v>0.2046221165714285</v>
       </c>
-      <c r="R22" t="n">
+      <c r="U22" t="n">
         <v>0.2619522340892465</v>
       </c>
-      <c r="S22" t="n">
+      <c r="V22" t="n">
         <v>0.1185852049427028</v>
       </c>
-      <c r="T22" t="n">
+      <c r="W22" t="n">
         <v>0.1224115124174072</v>
       </c>
-      <c r="U22" t="n">
+      <c r="X22" t="n">
         <v>0.01471401158005863</v>
       </c>
-      <c r="V22" t="n">
+      <c r="Y22" t="n">
         <v>0.1023360243809524</v>
       </c>
-      <c r="W22" t="n">
+      <c r="Z22" t="n">
         <v>0.1310080780297488</v>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>thread 2300680 (pt_autograd_0)</t>
-        </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -13924,102 +13924,102 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>thread 2300490 (python)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>(1, 128, 32, 32)</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>('float', None)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>(131072, 1024, 32, 1)</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>128.0</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="K23" t="n">
+      <c r="N23" t="n">
         <v>0.000656128</v>
       </c>
-      <c r="L23" t="n">
+      <c r="O23" t="n">
         <v>1.0029296875</v>
       </c>
-      <c r="M23" t="n">
+      <c r="P23" t="n">
         <v>0.623904576436222</v>
       </c>
-      <c r="N23" t="n">
+      <c r="Q23" t="n">
         <v>0.2440596457532344</v>
       </c>
-      <c r="O23" t="n">
+      <c r="R23" t="n">
         <v>0.2524941505275499</v>
       </c>
-      <c r="P23" t="n">
+      <c r="S23" t="n">
         <v>0.02904039043709479</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="T23" t="n">
         <v>0.2117356570979159</v>
       </c>
-      <c r="R23" t="n">
+      <c r="U23" t="n">
         <v>0.2679491296342374</v>
       </c>
-      <c r="S23" t="n">
+      <c r="V23" t="n">
         <v>0.1522699299088461</v>
       </c>
-      <c r="T23" t="n">
+      <c r="W23" t="n">
         <v>0.1575322560375147</v>
       </c>
-      <c r="U23" t="n">
+      <c r="X23" t="n">
         <v>0.01811843249519814</v>
       </c>
-      <c r="V23" t="n">
+      <c r="Y23" t="n">
         <v>0.1321028454581203</v>
       </c>
-      <c r="W23" t="n">
+      <c r="Z23" t="n">
         <v>0.1671746882309032</v>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>thread 2300490 (python)</t>
-        </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>

</xml_diff>